<commit_message>
Orçamento inclui link, perdido e reserva; recalcula funil e atendentes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dados-funil-leange-setembro.xlsx
+++ b/dados-funil-leange-setembro.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -581,34 +581,84 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Orçamentos abertos</t>
+          <t>Chegaram ao orçamento</t>
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>364</v>
+        <v>770</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
+          <t>% leads → orçamento</t>
+        </is>
+      </c>
+      <c r="B12" s="7">
+        <f>B11/B2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>% orçamento → reserva</t>
+        </is>
+      </c>
+      <c r="B13" s="7">
+        <f>B4/B11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Perdidos pós-orçamento (sem motivo)</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Orçamentos abertos</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
           <t>Orçamentos parados &gt; 7 dias</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n">
+      <c r="B16" s="3" t="n">
         <v>101</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+    <row r="17"/>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
         <is>
           <t>Receita em R$ arredondada a centenas (valores do dashboard).</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="8" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>Fonte: export Kommo, Funil de Vendas, leads criados 01–25/09/2026 (16h10). Taxas sobre leads criados até 20/09 salvo indicação.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>* % orçamento em aberto = só 'Orçamento enviado' e 'Link/dados'; não inclui perdidos pós-orçamento nem reservas.</t>
         </is>
       </c>
     </row>
@@ -623,12 +673,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
@@ -645,7 +695,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>% com orçamento</t>
+          <t>% orçamento em aberto*</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -779,10 +829,18 @@
       <c r="C9" s="11" t="n"/>
       <c r="D9" s="11" t="n"/>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
           <t>Fonte: export Kommo, Funil de Vendas, leads criados 01–25/09/2026 (16h10). Taxas sobre leads criados até 20/09 salvo indicação.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>* % orçamento em aberto = só 'Orçamento enviado' e 'Link/dados'; não inclui perdidos pós-orçamento nem reservas.</t>
         </is>
       </c>
     </row>
@@ -797,16 +855,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="27" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="27" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -822,25 +882,35 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>% com orçamento</t>
+          <t>% orçamento em aberto</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>% perdido pós-orçamento</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Reservas</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>% chegaram ao orçamento</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>% orçamento → reserva</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>% sumiram</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>% perdido sem motivo</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Reservas</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Receita (R$)</t>
         </is>
@@ -859,15 +929,23 @@
         <v>0.249</v>
       </c>
       <c r="D2" s="7" t="n">
+        <v>0.048</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="F2" s="7">
+        <f>C2+D2+E2/B2</f>
+        <v/>
+      </c>
+      <c r="G2" s="7">
+        <f>IF(F2=0,0,E2/(F2*B2))</f>
+        <v/>
+      </c>
+      <c r="H2" s="7" t="n">
         <v>0.601</v>
       </c>
-      <c r="E2" s="7" t="n">
-        <v>0.048</v>
-      </c>
-      <c r="F2" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="G2" s="6" t="n">
+      <c r="I2" s="6" t="n">
         <v>54000</v>
       </c>
     </row>
@@ -884,15 +962,23 @@
         <v>0.117</v>
       </c>
       <c r="D3" s="7" t="n">
+        <v>0.217</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="F3" s="7">
+        <f>C3+D3+E3/B3</f>
+        <v/>
+      </c>
+      <c r="G3" s="7">
+        <f>IF(F3=0,0,E3/(F3*B3))</f>
+        <v/>
+      </c>
+      <c r="H3" s="7" t="n">
         <v>0.5590000000000001</v>
       </c>
-      <c r="E3" s="7" t="n">
-        <v>0.217</v>
-      </c>
-      <c r="F3" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="G3" s="6" t="n">
+      <c r="I3" s="6" t="n">
         <v>67900</v>
       </c>
     </row>
@@ -909,15 +995,23 @@
         <v>0.045</v>
       </c>
       <c r="D4" s="7" t="n">
+        <v>0.337</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="F4" s="7">
+        <f>C4+D4+E4/B4</f>
+        <v/>
+      </c>
+      <c r="G4" s="7">
+        <f>IF(F4=0,0,E4/(F4*B4))</f>
+        <v/>
+      </c>
+      <c r="H4" s="7" t="n">
         <v>0.527</v>
       </c>
-      <c r="E4" s="7" t="n">
-        <v>0.337</v>
-      </c>
-      <c r="F4" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="G4" s="6" t="n">
+      <c r="I4" s="6" t="n">
         <v>27800</v>
       </c>
     </row>
@@ -934,15 +1028,23 @@
         <v>0.07099999999999999</v>
       </c>
       <c r="D5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="7">
+        <f>C5+D5+E5/B5</f>
+        <v/>
+      </c>
+      <c r="G5" s="7">
+        <f>IF(F5=0,0,E5/(F5*B5))</f>
+        <v/>
+      </c>
+      <c r="H5" s="7" t="n">
         <v>0.143</v>
       </c>
-      <c r="E5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" s="6" t="n">
+      <c r="I5" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -958,20 +1060,23 @@
       </c>
       <c r="C6" s="11" t="n"/>
       <c r="D6" s="11" t="n"/>
-      <c r="E6" s="11" t="n"/>
-      <c r="F6" s="10">
-        <f>SUM(F2:F5)</f>
-        <v/>
-      </c>
-      <c r="G6" s="12">
-        <f>SUM(G2:G5)</f>
-        <v/>
-      </c>
-    </row>
+      <c r="E6" s="10">
+        <f>SUM(E2:E5)</f>
+        <v/>
+      </c>
+      <c r="F6" s="11" t="n"/>
+      <c r="G6" s="11" t="n"/>
+      <c r="H6" s="11" t="n"/>
+      <c r="I6" s="12">
+        <f>SUM(I2:I5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>Nomes anonimizados. Atendente A sem leads novos desde 14/09.</t>
+          <t>Nomes anonimizados. Chegaram ao orçamento = em aberto + perdido pós-orçamento + reservas. Reservas contadas no mês inteiro (taxas sobre leads até 20/09).</t>
         </is>
       </c>
     </row>
@@ -979,6 +1084,13 @@
       <c r="A9" s="8" t="inlineStr">
         <is>
           <t>Fonte: export Kommo, Funil de Vendas, leads criados 01–25/09/2026 (16h10). Taxas sobre leads criados até 20/09 salvo indicação.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>* % orçamento em aberto = só 'Orçamento enviado' e 'Link/dados'; não inclui perdidos pós-orçamento nem reservas.</t>
         </is>
       </c>
     </row>
@@ -993,7 +1105,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1073,6 +1185,7 @@
         <v/>
       </c>
     </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
@@ -1084,6 +1197,13 @@
       <c r="A10" s="8" t="inlineStr">
         <is>
           <t>Fonte: export Kommo, Funil de Vendas, leads criados 01–25/09/2026 (16h10). Taxas sobre leads criados até 20/09 salvo indicação.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>* % orçamento em aberto = só 'Orçamento enviado' e 'Link/dados'; não inclui perdidos pós-orçamento nem reservas.</t>
         </is>
       </c>
     </row>
@@ -1098,7 +1218,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1183,11 +1303,11 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Receberam orçamento</t>
+          <t>Receberam orçamento (aberto, link, perdido ou reserva)</t>
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>384</v>
+        <v>770</v>
       </c>
       <c r="C5" s="7">
         <f>B5/$B$2</f>
@@ -1201,11 +1321,11 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Reserva a partir do funil</t>
+          <t>Reservas</t>
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="C6" s="7">
         <f>B6/$B$2</f>
@@ -1216,10 +1336,11 @@
         <v/>
       </c>
     </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>Funil reconstruído pela etapa atual de cada lead (export não traz histórico). As 18 reservas foram cadastradas fora do funil.</t>
+          <t>Funil pela etapa atual. Orçamento inclui Orçamento enviado (364), Link/dados (2), Finalizado/perdido (386) e Reserva Concluída (18). Reservas foram cadastradas como cards novos já ganhos.</t>
         </is>
       </c>
     </row>
@@ -1227,6 +1348,13 @@
       <c r="A9" s="8" t="inlineStr">
         <is>
           <t>Fonte: export Kommo, Funil de Vendas, leads criados 01–25/09/2026 (16h10). Taxas sobre leads criados até 20/09 salvo indicação.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>* % orçamento em aberto = só 'Orçamento enviado' e 'Link/dados'; não inclui perdidos pós-orçamento nem reservas.</t>
         </is>
       </c>
     </row>
@@ -1241,7 +1369,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1250,7 +1378,7 @@
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
@@ -1290,7 +1418,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>% com orçamento</t>
+          <t>% orçamento em aberto*</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -1490,10 +1618,18 @@
         <v/>
       </c>
     </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
           <t>Fonte: export Kommo, Funil de Vendas, leads criados 01–25/09/2026 (16h10). Taxas sobre leads criados até 20/09 salvo indicação.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>* % orçamento em aberto = só 'Orçamento enviado' e 'Link/dados'; não inclui perdidos pós-orçamento nem reservas.</t>
         </is>
       </c>
     </row>
@@ -1508,7 +1644,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2153,10 +2289,18 @@
         <v/>
       </c>
     </row>
+    <row r="28"/>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
           <t>Fonte: export Kommo, Funil de Vendas, leads criados 01–25/09/2026 (16h10). Taxas sobre leads criados até 20/09 salvo indicação.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="8" t="inlineStr">
+        <is>
+          <t>* % orçamento em aberto = só 'Orçamento enviado' e 'Link/dados'; não inclui perdidos pós-orçamento nem reservas.</t>
         </is>
       </c>
     </row>
@@ -2171,7 +2315,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2334,10 +2478,18 @@
       </c>
       <c r="C11" s="11" t="n"/>
     </row>
+    <row r="12"/>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
           <t>Fonte: export Kommo, Funil de Vendas, leads criados 01–25/09/2026 (16h10). Taxas sobre leads criados até 20/09 salvo indicação.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>* % orçamento em aberto = só 'Orçamento enviado' e 'Link/dados'; não inclui perdidos pós-orçamento nem reservas.</t>
         </is>
       </c>
     </row>
@@ -2352,13 +2504,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
@@ -2382,7 +2534,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>% com orçamento</t>
+          <t>% orçamento em aberto*</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -2526,6 +2678,7 @@
         <v>0</v>
       </c>
     </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
@@ -2537,6 +2690,13 @@
       <c r="A9" s="8" t="inlineStr">
         <is>
           <t>Fonte: export Kommo, Funil de Vendas, leads criados 01–25/09/2026 (16h10). Taxas sobre leads criados até 20/09 salvo indicação.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>* % orçamento em aberto = só 'Orçamento enviado' e 'Link/dados'; não inclui perdidos pós-orçamento nem reservas.</t>
         </is>
       </c>
     </row>
@@ -2551,14 +2711,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -2585,7 +2745,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>% com orçamento</t>
+          <t>% orçamento em aberto*</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -2724,6 +2884,7 @@
       <c r="E7" s="7" t="n"/>
       <c r="F7" s="7" t="n"/>
     </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
@@ -2735,6 +2896,13 @@
       <c r="A10" s="8" t="inlineStr">
         <is>
           <t>Fonte: export Kommo, Funil de Vendas, leads criados 01–25/09/2026 (16h10). Taxas sobre leads criados até 20/09 salvo indicação.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>* % orçamento em aberto = só 'Orçamento enviado' e 'Link/dados'; não inclui perdidos pós-orçamento nem reservas.</t>
         </is>
       </c>
     </row>
@@ -2749,13 +2917,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -2777,7 +2945,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>% com orçamento</t>
+          <t>% orçamento em aberto*</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -2877,10 +3045,18 @@
         <v>0.522</v>
       </c>
     </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
           <t>Fonte: export Kommo, Funil de Vendas, leads criados 01–25/09/2026 (16h10). Taxas sobre leads criados até 20/09 salvo indicação.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>* % orçamento em aberto = só 'Orçamento enviado' e 'Link/dados'; não inclui perdidos pós-orçamento nem reservas.</t>
         </is>
       </c>
     </row>
@@ -2895,12 +3071,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
@@ -2917,7 +3093,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>% com orçamento</t>
+          <t>% orçamento em aberto*</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -3003,10 +3179,18 @@
       <c r="C6" s="11" t="n"/>
       <c r="D6" s="11" t="n"/>
     </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
           <t>Fonte: export Kommo, Funil de Vendas, leads criados 01–25/09/2026 (16h10). Taxas sobre leads criados até 20/09 salvo indicação.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>* % orçamento em aberto = só 'Orçamento enviado' e 'Link/dados'; não inclui perdidos pós-orçamento nem reservas.</t>
         </is>
       </c>
     </row>

</xml_diff>